<commit_message>
Le salaire saisi est déjà net d'impôt sur le revenu
Le modèle appliquait un taux de 90 % au salaire mensuel, ce qui revenait à
prélever l'impôt une seconde fois : 3 400 € est le montant réellement
disponible, prélèvement à la source déjà déduit.

- Paramètre « Part du salaire conservée après IR » supprimé (21 paramètres).
- Le salaire entre tel quel : 3 400 €/mois, 40 800 €/an nets.
- Conséquences : revenu total 2027 de 63 078 € au lieu de 59 418 €, épargne
  cumulée sur 37 mois de 187 649 € au lieu de 175 069 €, et le net consultant
  n'égale plus le salaire qu'en juin 2028 au lieu d'avril — la barre est
  plus haute.
- Jalon « le revenu total double le salaire » remplacé : il était devenu
  l'exact équivalent de « net consultant = salaire ». À sa place, « le MRR
  net seul remplace le salaire » (janvier 2029).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheets/consultant-agent-ia-v2.xlsx
+++ b/sheets/consultant-agent-ia-v2.xlsx
@@ -3249,7 +3249,7 @@
         <v/>
       </c>
       <c r="I6" s="93">
-        <f>(((($C6*('Paramètres'!$C$21/5)*$D6)/12)/(1-$E6^(1/12)))*(1-(1-(1-(1-$E6^(1/12)))^37)/(37*(1-$E6^(1/12))))*$F6+(($C6*('Paramètres'!$C$21/5)*$D6)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$37</f>
+        <f>(((($C6*('Paramètres'!$C$21/5)*$D6)/12)/(1-$E6^(1/12)))*(1-(1-(1-(1-$E6^(1/12)))^37)/(37*(1-$E6^(1/12))))*$F6+(($C6*('Paramètres'!$C$21/5)*$D6)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$36</f>
         <v/>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
         <v/>
       </c>
       <c r="I7" s="93">
-        <f>(((($C7*('Paramètres'!$C$21/5)*$D7)/12)/(1-$E7^(1/12)))*(1-(1-(1-(1-$E7^(1/12)))^37)/(37*(1-$E7^(1/12))))*$F7+(($C7*('Paramètres'!$C$21/5)*$D7)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$37</f>
+        <f>(((($C7*('Paramètres'!$C$21/5)*$D7)/12)/(1-$E7^(1/12)))*(1-(1-(1-(1-$E7^(1/12)))^37)/(37*(1-$E7^(1/12))))*$F7+(($C7*('Paramètres'!$C$21/5)*$D7)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$36</f>
         <v/>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
         <v/>
       </c>
       <c r="I8" s="93">
-        <f>(((($C8*('Paramètres'!$C$21/5)*$D8)/12)/(1-$E8^(1/12)))*(1-(1-(1-(1-$E8^(1/12)))^37)/(37*(1-$E8^(1/12))))*$F8+(($C8*('Paramètres'!$C$21/5)*$D8)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$37</f>
+        <f>(((($C8*('Paramètres'!$C$21/5)*$D8)/12)/(1-$E8^(1/12)))*(1-(1-(1-(1-$E8^(1/12)))^37)/(37*(1-$E8^(1/12))))*$F8+(($C8*('Paramètres'!$C$21/5)*$D8)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$36</f>
         <v/>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
         <v/>
       </c>
       <c r="I9" s="93">
-        <f>(((($C9*('Paramètres'!$C$21/5)*$D9)/12)/(1-$E9^(1/12)))*(1-(1-(1-(1-$E9^(1/12)))^37)/(37*(1-$E9^(1/12))))*$F9+(($C9*('Paramètres'!$C$21/5)*$D9)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$37</f>
+        <f>(((($C9*('Paramètres'!$C$21/5)*$D9)/12)/(1-$E9^(1/12)))*(1-(1-(1-(1-$E9^(1/12)))^37)/(37*(1-$E9^(1/12))))*$F9+(($C9*('Paramètres'!$C$21/5)*$D9)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$36</f>
         <v/>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
         <v/>
       </c>
       <c r="I10" s="93">
-        <f>(((($C10*('Paramètres'!$C$21/5)*$D10)/12)/(1-$E10^(1/12)))*(1-(1-(1-(1-$E10^(1/12)))^37)/(37*(1-$E10^(1/12))))*$F10+(($C10*('Paramètres'!$C$21/5)*$D10)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$37</f>
+        <f>(((($C10*('Paramètres'!$C$21/5)*$D10)/12)/(1-$E10^(1/12)))*(1-(1-(1-(1-$E10^(1/12)))^37)/(37*(1-$E10^(1/12))))*$F10+(($C10*('Paramètres'!$C$21/5)*$D10)/12)*'Paramètres'!$C$8)*'Paramètres'!$C$36</f>
         <v/>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F45"/>
+  <dimension ref="B1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3826,7 +3826,7 @@
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Salaire net mensuel (avant IR)</t>
+          <t>Salaire mensuel net d'impôt (après IR)</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
@@ -3842,302 +3842,279 @@
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Salaire net versé, avant prélèvement à la source.</t>
+          <t>Montant réellement disponible chaque mois, prélèvement à la source déjà déduit.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Part du salaire conservée après IR</t>
-        </is>
-      </c>
-      <c r="C28" s="16" t="n">
-        <v>0.9</v>
+          <t>Jours travaillés par semaine (temps partiel)</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E28" s="17" t="n">
-        <v>0.9</v>
+          <t>j/sem</t>
+        </is>
+      </c>
+      <c r="E28" s="21" t="n">
+        <v>4</v>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>90 % correspond à 10 % de prélèvement à la source.</t>
+          <t>Contrat à temps partiel.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Jours travaillés par semaine (temps partiel)</t>
+          <t>Heures de présence par jour</t>
         </is>
       </c>
       <c r="C29" s="20" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>j/sem</t>
+          <t>h/j</t>
         </is>
       </c>
       <c r="E29" s="21" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Contrat à temps partiel.</t>
+          <t>Temps de présence contractuel.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Heures de présence par jour</t>
-        </is>
-      </c>
-      <c r="C30" s="20" t="n">
-        <v>8</v>
+          <t>Heures de travail cérébral réel par jour</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>3</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
           <t>h/j</t>
         </is>
       </c>
-      <c r="E30" s="21" t="n">
-        <v>8</v>
+      <c r="E30" s="15" t="n">
+        <v>3</v>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Temps de présence contractuel.</t>
+          <t>Production intellectuelle effective.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Heures de travail cérébral réel par jour</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="n">
-        <v>3</v>
+          <t>Semaines travaillées par an</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>44</v>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>h/j</t>
-        </is>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>3</v>
+          <t>sem/an</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>44</v>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>Production intellectuelle effective.</t>
+          <t>52 semaines moins congés et RTT.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Semaines travaillées par an</t>
-        </is>
-      </c>
-      <c r="C32" s="18" t="n">
-        <v>44</v>
+          <t>Jours de télétravail par semaine</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="n">
+        <v>1</v>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>sem/an</t>
-        </is>
-      </c>
-      <c r="E32" s="19" t="n">
-        <v>44</v>
+          <t>j/sem</t>
+        </is>
+      </c>
+      <c r="E32" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>52 semaines moins congés et RTT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Jours de télétravail par semaine</t>
-        </is>
-      </c>
-      <c r="C33" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>j/sem</t>
-        </is>
-      </c>
-      <c r="E33" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
           <t>Déduits des jours de présence sur site.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="8" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Fiscalité &amp; train de vie</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="B36" s="9" t="inlineStr">
+    <row r="35" ht="18" customHeight="1">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Paramètre</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>Défaut</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Rôle dans le modèle</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Part du CA consultant conservée (net IR)</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Cotisations + impôt sur le revenu + frais d'API des agents IA.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Part du CA consultant conservée (net IR)</t>
-        </is>
-      </c>
-      <c r="C37" s="16" t="n">
-        <v>0.5</v>
+          <t>Dépenses personnelles mensuelles</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>1800</v>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E37" s="17" t="n">
-        <v>0.5</v>
+          <t>€/mois</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="n">
+        <v>1800</v>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>Cotisations + impôt sur le revenu + frais d'API des agents IA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Dépenses personnelles mensuelles</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="n">
-        <v>1800</v>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>€/mois</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="n">
-        <v>1800</v>
-      </c>
-      <c r="F38" s="12" t="inlineStr">
-        <is>
           <t>Train de vie complet. Sert au calcul de l'épargne.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="8" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Horizon de projection</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="B41" s="9" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>Paramètre</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>Défaut</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>Rôle dans le modèle</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Année du premier mois projeté</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D41" s="12" t="inlineStr"/>
+      <c r="E41" s="19" t="n">
+        <v>2027</v>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Le tableau MRR démarre à ce mois et couvre 37 mois.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Année du premier mois projeté</t>
+          <t>Mois du premier mois projeté (1 = janvier)</t>
         </is>
       </c>
       <c r="C42" s="18" t="n">
-        <v>2027</v>
+        <v>1</v>
       </c>
       <c r="D42" s="12" t="inlineStr"/>
       <c r="E42" s="19" t="n">
-        <v>2027</v>
+        <v>1</v>
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>Le tableau MRR démarre à ce mois et couvre 37 mois.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>Mois du premier mois projeté (1 = janvier)</t>
-        </is>
-      </c>
-      <c r="C43" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="12" t="inlineStr"/>
-      <c r="E43" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
           <t>1 pour janvier. Le tableau va jusqu'à 01/2030 avec les valeurs par défaut.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="22" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="22" t="inlineStr">
         <is>
           <t>Colonne « Défaut » : valeur d'origine de l'étude, conservée pour référence.</t>
         </is>
@@ -4301,7 +4278,7 @@
         </is>
       </c>
       <c r="C11" s="23">
-        <f>'MRR mensuel'!$N$40*'Paramètres'!$C$37</f>
+        <f>'MRR mensuel'!$N$40*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -4402,7 +4379,7 @@
         </is>
       </c>
       <c r="F17" s="23">
-        <f>'Synthèse annuelle'!$D$6*'Paramètres'!$C$37</f>
+        <f>'Synthèse annuelle'!$D$6*'Paramètres'!$C$36</f>
         <v/>
       </c>
     </row>
@@ -4614,7 +4591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E45"/>
+  <dimension ref="B2:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5278,7 +5255,7 @@
         </is>
       </c>
       <c r="C39" s="33">
-        <f>'Hypothèses'!$C$38*'Paramètres'!$C$37</f>
+        <f>'Hypothèses'!$C$38*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="D39" s="12" t="inlineStr">
@@ -5328,7 +5305,7 @@
         </is>
       </c>
       <c r="C43" s="33">
-        <f>'Paramètres'!$C$27*'Paramètres'!$C$28</f>
+        <f>'Paramètres'!$C$27</f>
         <v/>
       </c>
       <c r="D43" s="12" t="inlineStr">
@@ -5338,7 +5315,7 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>salaire × taux_net_IR_salaire</t>
+          <t>paramètre : déjà net d'impôt</t>
         </is>
       </c>
     </row>
@@ -5360,27 +5337,6 @@
       <c r="E44" s="12" t="inlineStr">
         <is>
           <t>salaire_net_mensuel × 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="10" t="inlineStr">
-        <is>
-          <t>Salaire annuel net avant IR</t>
-        </is>
-      </c>
-      <c r="C45" s="33">
-        <f>'Paramètres'!$C$27*12</f>
-        <v/>
-      </c>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>€/an</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>salaire × 12</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5412,7 @@
         </is>
       </c>
       <c r="C7" s="34">
-        <f>'Paramètres'!$C$29*'Paramètres'!$C$30</f>
+        <f>'Paramètres'!$C$28*'Paramètres'!$C$29</f>
         <v/>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -5477,7 +5433,7 @@
         </is>
       </c>
       <c r="C8" s="34">
-        <f>'Paramètres'!$C$29*'Paramètres'!$C$31</f>
+        <f>'Paramètres'!$C$28*'Paramètres'!$C$30</f>
         <v/>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -5498,7 +5454,7 @@
         </is>
       </c>
       <c r="C9" s="35">
-        <f>'Temps &amp; capacité'!$C$7*'Paramètres'!$C$32</f>
+        <f>'Temps &amp; capacité'!$C$7*'Paramètres'!$C$31</f>
         <v/>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -5519,7 +5475,7 @@
         </is>
       </c>
       <c r="C10" s="35">
-        <f>'Temps &amp; capacité'!$C$8*'Paramètres'!$C$32</f>
+        <f>'Temps &amp; capacité'!$C$8*'Paramètres'!$C$31</f>
         <v/>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -5540,7 +5496,7 @@
         </is>
       </c>
       <c r="C11" s="38">
-        <f>'Paramètres'!$C$29*'Paramètres'!$C$32</f>
+        <f>'Paramètres'!$C$28*'Paramètres'!$C$31</f>
         <v/>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -5561,7 +5517,7 @@
         </is>
       </c>
       <c r="C12" s="38">
-        <f>('Paramètres'!$C$29-'Paramètres'!$C$33)*'Paramètres'!$C$32</f>
+        <f>('Paramètres'!$C$28-'Paramètres'!$C$32)*'Paramètres'!$C$31</f>
         <v/>
       </c>
       <c r="D12" s="12" t="inlineStr">
@@ -5582,7 +5538,7 @@
         </is>
       </c>
       <c r="C13" s="32">
-        <f>'Paramètres'!$C$31</f>
+        <f>'Paramètres'!$C$30</f>
         <v/>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -6149,7 +6105,7 @@
         </is>
       </c>
       <c r="C9" s="39">
-        <f>'Unit economics'!$C$8*'Paramètres'!$C$37</f>
+        <f>'Unit economics'!$C$8*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -6170,7 +6126,7 @@
         </is>
       </c>
       <c r="C10" s="39">
-        <f>'Unit economics'!$C$7*'Paramètres'!$C$37</f>
+        <f>'Unit economics'!$C$7*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -6480,7 +6436,7 @@
         </is>
       </c>
       <c r="C28" s="39">
-        <f>'Unit economics'!$C$26*'Paramètres'!$C$37</f>
+        <f>'Unit economics'!$C$26*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -6522,7 +6478,7 @@
         </is>
       </c>
       <c r="C30" s="33">
-        <f>'Unit economics'!$C$29*'Paramètres'!$C$37</f>
+        <f>'Unit economics'!$C$29*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -6805,7 +6761,7 @@
     </row>
     <row r="4">
       <c r="A4" s="44">
-        <f>DATE('Paramètres'!$C$42,'Paramètres'!$C$43,1)</f>
+        <f>DATE('Paramètres'!$C$41,'Paramètres'!$C$42,1)</f>
         <v/>
       </c>
       <c r="B4" s="45">
@@ -6832,15 +6788,15 @@
         <v/>
       </c>
       <c r="H4" s="47">
-        <f>F4*'Paramètres'!$C$37</f>
+        <f>F4*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I4" s="47">
-        <f>E4*'Paramètres'!$C$37</f>
+        <f>E4*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J4" s="47">
-        <f>G4*'Paramètres'!$C$37</f>
+        <f>G4*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K4" s="47">
@@ -6852,7 +6808,7 @@
         <v/>
       </c>
       <c r="M4" s="47">
-        <f>L4-'Paramètres'!$C$38</f>
+        <f>L4-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N4" s="47">
@@ -6906,15 +6862,15 @@
         <v/>
       </c>
       <c r="H5" s="54">
-        <f>F5*'Paramètres'!$C$37</f>
+        <f>F5*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I5" s="54">
-        <f>E5*'Paramètres'!$C$37</f>
+        <f>E5*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J5" s="54">
-        <f>G5*'Paramètres'!$C$37</f>
+        <f>G5*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K5" s="54">
@@ -6926,7 +6882,7 @@
         <v/>
       </c>
       <c r="M5" s="54">
-        <f>L5-'Paramètres'!$C$38</f>
+        <f>L5-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N5" s="54">
@@ -6980,15 +6936,15 @@
         <v/>
       </c>
       <c r="H6" s="47">
-        <f>F6*'Paramètres'!$C$37</f>
+        <f>F6*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I6" s="47">
-        <f>E6*'Paramètres'!$C$37</f>
+        <f>E6*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J6" s="47">
-        <f>G6*'Paramètres'!$C$37</f>
+        <f>G6*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K6" s="47">
@@ -7000,7 +6956,7 @@
         <v/>
       </c>
       <c r="M6" s="47">
-        <f>L6-'Paramètres'!$C$38</f>
+        <f>L6-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N6" s="47">
@@ -7054,15 +7010,15 @@
         <v/>
       </c>
       <c r="H7" s="54">
-        <f>F7*'Paramètres'!$C$37</f>
+        <f>F7*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I7" s="54">
-        <f>E7*'Paramètres'!$C$37</f>
+        <f>E7*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J7" s="54">
-        <f>G7*'Paramètres'!$C$37</f>
+        <f>G7*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K7" s="54">
@@ -7074,7 +7030,7 @@
         <v/>
       </c>
       <c r="M7" s="54">
-        <f>L7-'Paramètres'!$C$38</f>
+        <f>L7-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N7" s="54">
@@ -7128,15 +7084,15 @@
         <v/>
       </c>
       <c r="H8" s="47">
-        <f>F8*'Paramètres'!$C$37</f>
+        <f>F8*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I8" s="47">
-        <f>E8*'Paramètres'!$C$37</f>
+        <f>E8*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J8" s="47">
-        <f>G8*'Paramètres'!$C$37</f>
+        <f>G8*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K8" s="47">
@@ -7148,7 +7104,7 @@
         <v/>
       </c>
       <c r="M8" s="47">
-        <f>L8-'Paramètres'!$C$38</f>
+        <f>L8-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N8" s="47">
@@ -7202,15 +7158,15 @@
         <v/>
       </c>
       <c r="H9" s="54">
-        <f>F9*'Paramètres'!$C$37</f>
+        <f>F9*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I9" s="54">
-        <f>E9*'Paramètres'!$C$37</f>
+        <f>E9*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J9" s="54">
-        <f>G9*'Paramètres'!$C$37</f>
+        <f>G9*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K9" s="54">
@@ -7222,7 +7178,7 @@
         <v/>
       </c>
       <c r="M9" s="54">
-        <f>L9-'Paramètres'!$C$38</f>
+        <f>L9-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N9" s="54">
@@ -7276,15 +7232,15 @@
         <v/>
       </c>
       <c r="H10" s="47">
-        <f>F10*'Paramètres'!$C$37</f>
+        <f>F10*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I10" s="47">
-        <f>E10*'Paramètres'!$C$37</f>
+        <f>E10*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J10" s="47">
-        <f>G10*'Paramètres'!$C$37</f>
+        <f>G10*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K10" s="47">
@@ -7296,7 +7252,7 @@
         <v/>
       </c>
       <c r="M10" s="47">
-        <f>L10-'Paramètres'!$C$38</f>
+        <f>L10-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N10" s="47">
@@ -7350,15 +7306,15 @@
         <v/>
       </c>
       <c r="H11" s="54">
-        <f>F11*'Paramètres'!$C$37</f>
+        <f>F11*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I11" s="54">
-        <f>E11*'Paramètres'!$C$37</f>
+        <f>E11*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J11" s="54">
-        <f>G11*'Paramètres'!$C$37</f>
+        <f>G11*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K11" s="54">
@@ -7370,7 +7326,7 @@
         <v/>
       </c>
       <c r="M11" s="54">
-        <f>L11-'Paramètres'!$C$38</f>
+        <f>L11-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N11" s="54">
@@ -7424,15 +7380,15 @@
         <v/>
       </c>
       <c r="H12" s="47">
-        <f>F12*'Paramètres'!$C$37</f>
+        <f>F12*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I12" s="47">
-        <f>E12*'Paramètres'!$C$37</f>
+        <f>E12*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J12" s="47">
-        <f>G12*'Paramètres'!$C$37</f>
+        <f>G12*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K12" s="47">
@@ -7444,7 +7400,7 @@
         <v/>
       </c>
       <c r="M12" s="47">
-        <f>L12-'Paramètres'!$C$38</f>
+        <f>L12-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N12" s="47">
@@ -7498,15 +7454,15 @@
         <v/>
       </c>
       <c r="H13" s="54">
-        <f>F13*'Paramètres'!$C$37</f>
+        <f>F13*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I13" s="54">
-        <f>E13*'Paramètres'!$C$37</f>
+        <f>E13*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J13" s="54">
-        <f>G13*'Paramètres'!$C$37</f>
+        <f>G13*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K13" s="54">
@@ -7518,7 +7474,7 @@
         <v/>
       </c>
       <c r="M13" s="54">
-        <f>L13-'Paramètres'!$C$38</f>
+        <f>L13-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N13" s="54">
@@ -7572,15 +7528,15 @@
         <v/>
       </c>
       <c r="H14" s="47">
-        <f>F14*'Paramètres'!$C$37</f>
+        <f>F14*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I14" s="47">
-        <f>E14*'Paramètres'!$C$37</f>
+        <f>E14*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J14" s="47">
-        <f>G14*'Paramètres'!$C$37</f>
+        <f>G14*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K14" s="47">
@@ -7592,7 +7548,7 @@
         <v/>
       </c>
       <c r="M14" s="47">
-        <f>L14-'Paramètres'!$C$38</f>
+        <f>L14-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N14" s="47">
@@ -7646,15 +7602,15 @@
         <v/>
       </c>
       <c r="H15" s="54">
-        <f>F15*'Paramètres'!$C$37</f>
+        <f>F15*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I15" s="54">
-        <f>E15*'Paramètres'!$C$37</f>
+        <f>E15*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J15" s="54">
-        <f>G15*'Paramètres'!$C$37</f>
+        <f>G15*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K15" s="54">
@@ -7666,7 +7622,7 @@
         <v/>
       </c>
       <c r="M15" s="54">
-        <f>L15-'Paramètres'!$C$38</f>
+        <f>L15-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N15" s="54">
@@ -7720,15 +7676,15 @@
         <v/>
       </c>
       <c r="H16" s="47">
-        <f>F16*'Paramètres'!$C$37</f>
+        <f>F16*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I16" s="47">
-        <f>E16*'Paramètres'!$C$37</f>
+        <f>E16*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J16" s="47">
-        <f>G16*'Paramètres'!$C$37</f>
+        <f>G16*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K16" s="47">
@@ -7740,7 +7696,7 @@
         <v/>
       </c>
       <c r="M16" s="47">
-        <f>L16-'Paramètres'!$C$38</f>
+        <f>L16-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N16" s="47">
@@ -7794,15 +7750,15 @@
         <v/>
       </c>
       <c r="H17" s="54">
-        <f>F17*'Paramètres'!$C$37</f>
+        <f>F17*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I17" s="54">
-        <f>E17*'Paramètres'!$C$37</f>
+        <f>E17*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J17" s="54">
-        <f>G17*'Paramètres'!$C$37</f>
+        <f>G17*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K17" s="54">
@@ -7814,7 +7770,7 @@
         <v/>
       </c>
       <c r="M17" s="54">
-        <f>L17-'Paramètres'!$C$38</f>
+        <f>L17-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N17" s="54">
@@ -7868,15 +7824,15 @@
         <v/>
       </c>
       <c r="H18" s="47">
-        <f>F18*'Paramètres'!$C$37</f>
+        <f>F18*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I18" s="47">
-        <f>E18*'Paramètres'!$C$37</f>
+        <f>E18*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J18" s="47">
-        <f>G18*'Paramètres'!$C$37</f>
+        <f>G18*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K18" s="47">
@@ -7888,7 +7844,7 @@
         <v/>
       </c>
       <c r="M18" s="47">
-        <f>L18-'Paramètres'!$C$38</f>
+        <f>L18-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N18" s="47">
@@ -7942,15 +7898,15 @@
         <v/>
       </c>
       <c r="H19" s="54">
-        <f>F19*'Paramètres'!$C$37</f>
+        <f>F19*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I19" s="54">
-        <f>E19*'Paramètres'!$C$37</f>
+        <f>E19*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J19" s="54">
-        <f>G19*'Paramètres'!$C$37</f>
+        <f>G19*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K19" s="54">
@@ -7962,7 +7918,7 @@
         <v/>
       </c>
       <c r="M19" s="54">
-        <f>L19-'Paramètres'!$C$38</f>
+        <f>L19-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N19" s="54">
@@ -8016,15 +7972,15 @@
         <v/>
       </c>
       <c r="H20" s="47">
-        <f>F20*'Paramètres'!$C$37</f>
+        <f>F20*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I20" s="47">
-        <f>E20*'Paramètres'!$C$37</f>
+        <f>E20*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J20" s="47">
-        <f>G20*'Paramètres'!$C$37</f>
+        <f>G20*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K20" s="47">
@@ -8036,7 +7992,7 @@
         <v/>
       </c>
       <c r="M20" s="47">
-        <f>L20-'Paramètres'!$C$38</f>
+        <f>L20-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N20" s="47">
@@ -8090,15 +8046,15 @@
         <v/>
       </c>
       <c r="H21" s="54">
-        <f>F21*'Paramètres'!$C$37</f>
+        <f>F21*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I21" s="54">
-        <f>E21*'Paramètres'!$C$37</f>
+        <f>E21*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J21" s="54">
-        <f>G21*'Paramètres'!$C$37</f>
+        <f>G21*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K21" s="54">
@@ -8110,7 +8066,7 @@
         <v/>
       </c>
       <c r="M21" s="54">
-        <f>L21-'Paramètres'!$C$38</f>
+        <f>L21-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N21" s="54">
@@ -8164,15 +8120,15 @@
         <v/>
       </c>
       <c r="H22" s="47">
-        <f>F22*'Paramètres'!$C$37</f>
+        <f>F22*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I22" s="47">
-        <f>E22*'Paramètres'!$C$37</f>
+        <f>E22*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J22" s="47">
-        <f>G22*'Paramètres'!$C$37</f>
+        <f>G22*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K22" s="47">
@@ -8184,7 +8140,7 @@
         <v/>
       </c>
       <c r="M22" s="47">
-        <f>L22-'Paramètres'!$C$38</f>
+        <f>L22-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N22" s="47">
@@ -8238,15 +8194,15 @@
         <v/>
       </c>
       <c r="H23" s="54">
-        <f>F23*'Paramètres'!$C$37</f>
+        <f>F23*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I23" s="54">
-        <f>E23*'Paramètres'!$C$37</f>
+        <f>E23*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J23" s="54">
-        <f>G23*'Paramètres'!$C$37</f>
+        <f>G23*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K23" s="54">
@@ -8258,7 +8214,7 @@
         <v/>
       </c>
       <c r="M23" s="54">
-        <f>L23-'Paramètres'!$C$38</f>
+        <f>L23-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N23" s="54">
@@ -8312,15 +8268,15 @@
         <v/>
       </c>
       <c r="H24" s="47">
-        <f>F24*'Paramètres'!$C$37</f>
+        <f>F24*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I24" s="47">
-        <f>E24*'Paramètres'!$C$37</f>
+        <f>E24*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J24" s="47">
-        <f>G24*'Paramètres'!$C$37</f>
+        <f>G24*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K24" s="47">
@@ -8332,7 +8288,7 @@
         <v/>
       </c>
       <c r="M24" s="47">
-        <f>L24-'Paramètres'!$C$38</f>
+        <f>L24-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N24" s="47">
@@ -8386,15 +8342,15 @@
         <v/>
       </c>
       <c r="H25" s="54">
-        <f>F25*'Paramètres'!$C$37</f>
+        <f>F25*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I25" s="54">
-        <f>E25*'Paramètres'!$C$37</f>
+        <f>E25*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J25" s="54">
-        <f>G25*'Paramètres'!$C$37</f>
+        <f>G25*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K25" s="54">
@@ -8406,7 +8362,7 @@
         <v/>
       </c>
       <c r="M25" s="54">
-        <f>L25-'Paramètres'!$C$38</f>
+        <f>L25-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N25" s="54">
@@ -8460,15 +8416,15 @@
         <v/>
       </c>
       <c r="H26" s="47">
-        <f>F26*'Paramètres'!$C$37</f>
+        <f>F26*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I26" s="47">
-        <f>E26*'Paramètres'!$C$37</f>
+        <f>E26*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J26" s="47">
-        <f>G26*'Paramètres'!$C$37</f>
+        <f>G26*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K26" s="47">
@@ -8480,7 +8436,7 @@
         <v/>
       </c>
       <c r="M26" s="47">
-        <f>L26-'Paramètres'!$C$38</f>
+        <f>L26-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N26" s="47">
@@ -8534,15 +8490,15 @@
         <v/>
       </c>
       <c r="H27" s="54">
-        <f>F27*'Paramètres'!$C$37</f>
+        <f>F27*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I27" s="54">
-        <f>E27*'Paramètres'!$C$37</f>
+        <f>E27*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J27" s="54">
-        <f>G27*'Paramètres'!$C$37</f>
+        <f>G27*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K27" s="54">
@@ -8554,7 +8510,7 @@
         <v/>
       </c>
       <c r="M27" s="54">
-        <f>L27-'Paramètres'!$C$38</f>
+        <f>L27-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N27" s="54">
@@ -8608,15 +8564,15 @@
         <v/>
       </c>
       <c r="H28" s="47">
-        <f>F28*'Paramètres'!$C$37</f>
+        <f>F28*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I28" s="47">
-        <f>E28*'Paramètres'!$C$37</f>
+        <f>E28*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J28" s="47">
-        <f>G28*'Paramètres'!$C$37</f>
+        <f>G28*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K28" s="47">
@@ -8628,7 +8584,7 @@
         <v/>
       </c>
       <c r="M28" s="47">
-        <f>L28-'Paramètres'!$C$38</f>
+        <f>L28-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N28" s="47">
@@ -8682,15 +8638,15 @@
         <v/>
       </c>
       <c r="H29" s="54">
-        <f>F29*'Paramètres'!$C$37</f>
+        <f>F29*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I29" s="54">
-        <f>E29*'Paramètres'!$C$37</f>
+        <f>E29*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J29" s="54">
-        <f>G29*'Paramètres'!$C$37</f>
+        <f>G29*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K29" s="54">
@@ -8702,7 +8658,7 @@
         <v/>
       </c>
       <c r="M29" s="54">
-        <f>L29-'Paramètres'!$C$38</f>
+        <f>L29-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N29" s="54">
@@ -8756,15 +8712,15 @@
         <v/>
       </c>
       <c r="H30" s="47">
-        <f>F30*'Paramètres'!$C$37</f>
+        <f>F30*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I30" s="47">
-        <f>E30*'Paramètres'!$C$37</f>
+        <f>E30*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J30" s="47">
-        <f>G30*'Paramètres'!$C$37</f>
+        <f>G30*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K30" s="47">
@@ -8776,7 +8732,7 @@
         <v/>
       </c>
       <c r="M30" s="47">
-        <f>L30-'Paramètres'!$C$38</f>
+        <f>L30-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N30" s="47">
@@ -8830,15 +8786,15 @@
         <v/>
       </c>
       <c r="H31" s="54">
-        <f>F31*'Paramètres'!$C$37</f>
+        <f>F31*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I31" s="54">
-        <f>E31*'Paramètres'!$C$37</f>
+        <f>E31*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J31" s="54">
-        <f>G31*'Paramètres'!$C$37</f>
+        <f>G31*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K31" s="54">
@@ -8850,7 +8806,7 @@
         <v/>
       </c>
       <c r="M31" s="54">
-        <f>L31-'Paramètres'!$C$38</f>
+        <f>L31-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N31" s="54">
@@ -8904,15 +8860,15 @@
         <v/>
       </c>
       <c r="H32" s="47">
-        <f>F32*'Paramètres'!$C$37</f>
+        <f>F32*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I32" s="47">
-        <f>E32*'Paramètres'!$C$37</f>
+        <f>E32*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J32" s="47">
-        <f>G32*'Paramètres'!$C$37</f>
+        <f>G32*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K32" s="47">
@@ -8924,7 +8880,7 @@
         <v/>
       </c>
       <c r="M32" s="47">
-        <f>L32-'Paramètres'!$C$38</f>
+        <f>L32-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N32" s="47">
@@ -8978,15 +8934,15 @@
         <v/>
       </c>
       <c r="H33" s="54">
-        <f>F33*'Paramètres'!$C$37</f>
+        <f>F33*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I33" s="54">
-        <f>E33*'Paramètres'!$C$37</f>
+        <f>E33*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J33" s="54">
-        <f>G33*'Paramètres'!$C$37</f>
+        <f>G33*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K33" s="54">
@@ -8998,7 +8954,7 @@
         <v/>
       </c>
       <c r="M33" s="54">
-        <f>L33-'Paramètres'!$C$38</f>
+        <f>L33-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N33" s="54">
@@ -9052,15 +9008,15 @@
         <v/>
       </c>
       <c r="H34" s="47">
-        <f>F34*'Paramètres'!$C$37</f>
+        <f>F34*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I34" s="47">
-        <f>E34*'Paramètres'!$C$37</f>
+        <f>E34*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J34" s="47">
-        <f>G34*'Paramètres'!$C$37</f>
+        <f>G34*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K34" s="47">
@@ -9072,7 +9028,7 @@
         <v/>
       </c>
       <c r="M34" s="47">
-        <f>L34-'Paramètres'!$C$38</f>
+        <f>L34-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N34" s="47">
@@ -9126,15 +9082,15 @@
         <v/>
       </c>
       <c r="H35" s="54">
-        <f>F35*'Paramètres'!$C$37</f>
+        <f>F35*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I35" s="54">
-        <f>E35*'Paramètres'!$C$37</f>
+        <f>E35*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J35" s="54">
-        <f>G35*'Paramètres'!$C$37</f>
+        <f>G35*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K35" s="54">
@@ -9146,7 +9102,7 @@
         <v/>
       </c>
       <c r="M35" s="54">
-        <f>L35-'Paramètres'!$C$38</f>
+        <f>L35-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N35" s="54">
@@ -9200,15 +9156,15 @@
         <v/>
       </c>
       <c r="H36" s="47">
-        <f>F36*'Paramètres'!$C$37</f>
+        <f>F36*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I36" s="47">
-        <f>E36*'Paramètres'!$C$37</f>
+        <f>E36*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J36" s="47">
-        <f>G36*'Paramètres'!$C$37</f>
+        <f>G36*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K36" s="47">
@@ -9220,7 +9176,7 @@
         <v/>
       </c>
       <c r="M36" s="47">
-        <f>L36-'Paramètres'!$C$38</f>
+        <f>L36-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N36" s="47">
@@ -9274,15 +9230,15 @@
         <v/>
       </c>
       <c r="H37" s="54">
-        <f>F37*'Paramètres'!$C$37</f>
+        <f>F37*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I37" s="54">
-        <f>E37*'Paramètres'!$C$37</f>
+        <f>E37*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J37" s="54">
-        <f>G37*'Paramètres'!$C$37</f>
+        <f>G37*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K37" s="54">
@@ -9294,7 +9250,7 @@
         <v/>
       </c>
       <c r="M37" s="54">
-        <f>L37-'Paramètres'!$C$38</f>
+        <f>L37-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N37" s="54">
@@ -9348,15 +9304,15 @@
         <v/>
       </c>
       <c r="H38" s="47">
-        <f>F38*'Paramètres'!$C$37</f>
+        <f>F38*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I38" s="47">
-        <f>E38*'Paramètres'!$C$37</f>
+        <f>E38*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J38" s="47">
-        <f>G38*'Paramètres'!$C$37</f>
+        <f>G38*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K38" s="47">
@@ -9368,7 +9324,7 @@
         <v/>
       </c>
       <c r="M38" s="47">
-        <f>L38-'Paramètres'!$C$38</f>
+        <f>L38-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N38" s="47">
@@ -9422,15 +9378,15 @@
         <v/>
       </c>
       <c r="H39" s="54">
-        <f>F39*'Paramètres'!$C$37</f>
+        <f>F39*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I39" s="54">
-        <f>E39*'Paramètres'!$C$37</f>
+        <f>E39*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J39" s="54">
-        <f>G39*'Paramètres'!$C$37</f>
+        <f>G39*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K39" s="54">
@@ -9442,7 +9398,7 @@
         <v/>
       </c>
       <c r="M39" s="54">
-        <f>L39-'Paramètres'!$C$38</f>
+        <f>L39-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N39" s="54">
@@ -9496,15 +9452,15 @@
         <v/>
       </c>
       <c r="H40" s="47">
-        <f>F40*'Paramètres'!$C$37</f>
+        <f>F40*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="I40" s="47">
-        <f>E40*'Paramètres'!$C$37</f>
+        <f>E40*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="J40" s="47">
-        <f>G40*'Paramètres'!$C$37</f>
+        <f>G40*'Paramètres'!$C$36</f>
         <v/>
       </c>
       <c r="K40" s="47">
@@ -9516,7 +9472,7 @@
         <v/>
       </c>
       <c r="M40" s="47">
-        <f>L40-'Paramètres'!$C$38</f>
+        <f>L40-'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="N40" s="47">
@@ -9732,7 +9688,7 @@
     </row>
     <row r="5">
       <c r="A5" s="38">
-        <f>'Paramètres'!$C$42</f>
+        <f>'Paramètres'!$C$41</f>
         <v/>
       </c>
       <c r="B5" s="63">
@@ -9768,7 +9724,7 @@
         <v/>
       </c>
       <c r="J5" s="47">
-        <f>B5*'Paramètres'!$C$38</f>
+        <f>B5*'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="K5" s="47">
@@ -9798,7 +9754,7 @@
     </row>
     <row r="6">
       <c r="A6" s="68">
-        <f>'Paramètres'!$C$42+1</f>
+        <f>'Paramètres'!$C$41+1</f>
         <v/>
       </c>
       <c r="B6" s="69">
@@ -9834,7 +9790,7 @@
         <v/>
       </c>
       <c r="J6" s="54">
-        <f>B6*'Paramètres'!$C$38</f>
+        <f>B6*'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="K6" s="54">
@@ -9864,7 +9820,7 @@
     </row>
     <row r="7">
       <c r="A7" s="38">
-        <f>'Paramètres'!$C$42+2</f>
+        <f>'Paramètres'!$C$41+2</f>
         <v/>
       </c>
       <c r="B7" s="63">
@@ -9900,7 +9856,7 @@
         <v/>
       </c>
       <c r="J7" s="47">
-        <f>B7*'Paramètres'!$C$38</f>
+        <f>B7*'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="K7" s="47">
@@ -9930,7 +9886,7 @@
     </row>
     <row r="8">
       <c r="A8" s="68">
-        <f>'Paramètres'!$C$42+3</f>
+        <f>'Paramètres'!$C$41+3</f>
         <v/>
       </c>
       <c r="B8" s="69">
@@ -9966,7 +9922,7 @@
         <v/>
       </c>
       <c r="J8" s="54">
-        <f>B8*'Paramètres'!$C$38</f>
+        <f>B8*'Paramètres'!$C$37</f>
         <v/>
       </c>
       <c r="K8" s="54">
@@ -10150,15 +10106,15 @@
         </is>
       </c>
       <c r="D7" s="80">
-        <f>IFERROR(INDEX('MRR mensuel'!$A$4:$A$40,MATCH(TRUE,('MRR mensuel'!$J$4:$J$40&gt;='Paramètres'!$C$38),0)),"hors horizon")</f>
+        <f>IFERROR(INDEX('MRR mensuel'!$A$4:$A$40,MATCH(TRUE,('MRR mensuel'!$J$4:$J$40&gt;='Paramètres'!$C$37),0)),"hors horizon")</f>
         <v/>
       </c>
       <c r="E7" s="81">
-        <f>IFERROR("M+"&amp;MATCH(TRUE,('MRR mensuel'!$J$4:$J$40&gt;='Paramètres'!$C$38),0),"—")</f>
+        <f>IFERROR("M+"&amp;MATCH(TRUE,('MRR mensuel'!$J$4:$J$40&gt;='Paramètres'!$C$37),0),"—")</f>
         <v/>
       </c>
       <c r="F7" s="33">
-        <f>IFERROR(INDEX('MRR mensuel'!$F$4:$F$40,MATCH(TRUE,('MRR mensuel'!$J$4:$J$40&gt;='Paramètres'!$C$38),0)),"—")</f>
+        <f>IFERROR(INDEX('MRR mensuel'!$F$4:$F$40,MATCH(TRUE,('MRR mensuel'!$J$4:$J$40&gt;='Paramètres'!$C$37),0)),"—")</f>
         <v/>
       </c>
     </row>
@@ -10246,39 +10202,39 @@
         </is>
       </c>
       <c r="D11" s="80">
-        <f>IFERROR(INDEX('MRR mensuel'!$A$4:$A$40,MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Paramètres'!$C$38),0)),"hors horizon")</f>
+        <f>IFERROR(INDEX('MRR mensuel'!$A$4:$A$40,MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Paramètres'!$C$37),0)),"hors horizon")</f>
         <v/>
       </c>
       <c r="E11" s="81">
-        <f>IFERROR("M+"&amp;MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Paramètres'!$C$38),0),"—")</f>
+        <f>IFERROR("M+"&amp;MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Paramètres'!$C$37),0),"—")</f>
         <v/>
       </c>
       <c r="F11" s="33">
-        <f>IFERROR(INDEX('MRR mensuel'!$F$4:$F$40,MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Paramètres'!$C$38),0)),"—")</f>
+        <f>IFERROR(INDEX('MRR mensuel'!$F$4:$F$40,MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Paramètres'!$C$37),0)),"—")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Le revenu total double le salaire net</t>
+          <t>Le MRR net seul remplace le salaire</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>revenu total ≥ 2 × salaire net</t>
+          <t>net MRR ≥ salaire net</t>
         </is>
       </c>
       <c r="D12" s="80">
-        <f>IFERROR(INDEX('MRR mensuel'!$A$4:$A$40,MATCH(TRUE,('MRR mensuel'!$L$4:$L$40&gt;=2*'Hypothèses'!$C$43),0)),"hors horizon")</f>
+        <f>IFERROR(INDEX('MRR mensuel'!$A$4:$A$40,MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Hypothèses'!$C$43),0)),"hors horizon")</f>
         <v/>
       </c>
       <c r="E12" s="81">
-        <f>IFERROR("M+"&amp;MATCH(TRUE,('MRR mensuel'!$L$4:$L$40&gt;=2*'Hypothèses'!$C$43),0),"—")</f>
+        <f>IFERROR("M+"&amp;MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Hypothèses'!$C$43),0),"—")</f>
         <v/>
       </c>
       <c r="F12" s="33">
-        <f>IFERROR(INDEX('MRR mensuel'!$F$4:$F$40,MATCH(TRUE,('MRR mensuel'!$L$4:$L$40&gt;=2*'Hypothèses'!$C$43),0)),"—")</f>
+        <f>IFERROR(INDEX('MRR mensuel'!$F$4:$F$40,MATCH(TRUE,('MRR mensuel'!$H$4:$H$40&gt;='Hypothèses'!$C$43),0)),"—")</f>
         <v/>
       </c>
     </row>

</xml_diff>